<commit_message>
week 2 homework part 1
</commit_message>
<xml_diff>
--- a/Excel/Woche2.xlsx
+++ b/Excel/Woche2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\DSI\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11562A32-9769-4871-8738-A19A8C5327B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A51FBD3-05B2-4670-ADE3-868923A0B405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0C427123-316F-40A9-A3DF-49E52740271D}"/>
   </bookViews>
@@ -485,7 +485,9 @@
     <c:title>
       <c:overlay val="0"/>
       <c:spPr>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="accent1"/>
+        </a:solidFill>
         <a:ln>
           <a:noFill/>
         </a:ln>
@@ -496,13 +498,19 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
                 </a:schemeClr>
               </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+                  <a:prstClr val="black">
+                    <a:alpha val="40000"/>
+                  </a:prstClr>
+                </a:outerShdw>
+              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -534,13 +542,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -653,13 +690,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent2">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent2">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -765,8 +831,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
+        <c:gapWidth val="100"/>
+        <c:overlap val="-24"/>
         <c:axId val="2115884496"/>
         <c:axId val="2115882096"/>
       </c:barChart>
@@ -777,17 +843,46 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="lt1">
+                      <a:lumMod val="85000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
+              <a:schemeClr val="lt1">
+                <a:lumMod val="95000"/>
+                <a:alpha val="54000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -801,9 +896,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -832,9 +926,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="95000"/>
+                  <a:alpha val="10000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -842,6 +936,35 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="lt1">
+                      <a:lumMod val="85000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -860,9 +983,8 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
+                  <a:schemeClr val="lt1">
+                    <a:lumMod val="85000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
@@ -902,9 +1024,8 @@
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
@@ -921,17 +1042,28 @@
     <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
+    <a:gradFill flip="none" rotWithShape="1">
+      <a:gsLst>
+        <a:gs pos="0">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:gs>
+        <a:gs pos="100000">
+          <a:schemeClr val="dk1">
+            <a:lumMod val="85000"/>
+            <a:lumOff val="15000"/>
+          </a:schemeClr>
+        </a:gs>
+      </a:gsLst>
+      <a:path path="circle">
+        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+      </a:path>
+      <a:tileRect/>
+    </a:gradFill>
+    <a:ln>
+      <a:noFill/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -3015,35 +3147,33 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="209">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
   </cs:axisTitle>
   <cs:categoryAxis>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3051,26 +3181,34 @@
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:gradFill flip="none" rotWithShape="1">
+        <a:gsLst>
+          <a:gs pos="0">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="65000"/>
+              <a:lumOff val="35000"/>
+            </a:schemeClr>
+          </a:gs>
+          <a:gs pos="100000">
+            <a:schemeClr val="dk1">
+              <a:lumMod val="85000"/>
+              <a:lumOff val="15000"/>
+            </a:schemeClr>
+          </a:gs>
+        </a:gsLst>
+        <a:path path="circle">
+          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+        </a:path>
+        <a:tileRect/>
+      </a:gradFill>
     </cs:spPr>
     <cs:defRPr sz="1000" kern="1200"/>
   </cs:chartArea>
@@ -3079,9 +3217,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3100,14 +3237,6 @@
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -3116,35 +3245,35 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="34925" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -3156,30 +3285,31 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -3195,21 +3325,18 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3219,20 +3346,20 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -3243,17 +3370,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -3262,14 +3389,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3281,28 +3407,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
   </cs:floor>
   <cs:gridlineMajor>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="10000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3314,17 +3434,16 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="5000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:gridlineMinor>
@@ -3333,17 +3452,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:hiLoLine>
@@ -3352,17 +3471,16 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:leaderLine>
@@ -3371,27 +3489,26 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:plotArea3D>
   <cs:seriesAxis>
@@ -3399,11 +3516,21 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
@@ -3411,14 +3538,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3430,12 +3557,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="95000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
+      <a:effectLst>
+        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
+          <a:prstClr val="black">
+            <a:alpha val="40000"/>
+          </a:prstClr>
+        </a:outerShdw>
+      </a:effectLst>
+    </cs:defRPr>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -3444,14 +3578,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:prstDash val="sysDot"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -3460,9 +3593,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3472,7 +3604,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -3480,9 +3612,9 @@
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="95000"/>
+            <a:alpha val="54000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -3493,9 +3625,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
+      <a:schemeClr val="lt1">
+        <a:lumMod val="85000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
@@ -3505,14 +3636,8 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>

</xml_diff>